<commit_message>
Update Wyscout report pages in Excel
</commit_message>
<xml_diff>
--- a/team_stats_perth.xlsx
+++ b/team_stats_perth.xlsx
@@ -12658,13 +12658,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="B1:C1"/>
     <mergeCell ref="AC1:AR1"/>
     <mergeCell ref="BM1:BN1"/>
     <mergeCell ref="D1:J1"/>
     <mergeCell ref="K1:T1"/>
     <mergeCell ref="AS1:BL1"/>
-    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="U1:AA1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização semanal — Round 13
</commit_message>
<xml_diff>
--- a/team_stats_perth.xlsx
+++ b/team_stats_perth.xlsx
@@ -7820,7 +7820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA27"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8008,63 +8008,63 @@
         <v>28.57</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>283</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>63.96</v>
       </c>
       <c r="P2" t="n">
-        <v>283</v>
+        <v>37.64</v>
       </c>
       <c r="Q2" t="n">
-        <v>181</v>
+        <v>126</v>
       </c>
       <c r="R2" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="S2" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="T2" t="n">
+        <v>62</v>
+      </c>
+      <c r="U2" t="n">
+        <v>88</v>
+      </c>
+      <c r="V2" t="n">
+        <v>44</v>
+      </c>
+      <c r="W2" t="n">
+        <v>30</v>
+      </c>
+      <c r="X2" t="n">
+        <v>14</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>237</v>
+      </c>
+      <c r="Z2" t="n">
         <v>126</v>
       </c>
-      <c r="U2" t="n">
-        <v>16</v>
-      </c>
-      <c r="V2" t="n">
-        <v>48</v>
-      </c>
-      <c r="W2" t="n">
-        <v>62</v>
-      </c>
-      <c r="X2" t="n">
-        <v>88</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>44</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>30</v>
-      </c>
       <c r="AA2" t="n">
-        <v>14</v>
+        <v>53.16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Perth - Fremantle City 2:1</t>
+          <t>Balcatta - Perth 0:1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -8073,91 +8073,91 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fremantle City</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-4-2 (100.0%)</t>
+          <t>4-1-4-1 (100.0%)</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1.24</v>
+        <v>0.66</v>
       </c>
       <c r="J3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L3" t="n">
-        <v>25</v>
+        <v>46.15</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>366</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>249</v>
       </c>
       <c r="O3" t="n">
-        <v>3</v>
+        <v>68.03</v>
       </c>
       <c r="P3" t="n">
-        <v>464</v>
+        <v>44.6</v>
       </c>
       <c r="Q3" t="n">
-        <v>364</v>
+        <v>136</v>
       </c>
       <c r="R3" t="n">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="S3" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="T3" t="n">
-        <v>133</v>
+        <v>74</v>
       </c>
       <c r="U3" t="n">
-        <v>25</v>
+        <v>99</v>
       </c>
       <c r="V3" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="W3" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="X3" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="Y3" t="n">
-        <v>34</v>
+        <v>215</v>
       </c>
       <c r="Z3" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="AA3" t="n">
-        <v>17</v>
+        <v>46.51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Balcatta - Perth 0:1</t>
+          <t>Perth - West NTC 3:0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -8166,7 +8166,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -8175,82 +8175,82 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-1-4-1 (100.0%)</t>
+          <t>4-2-3-1 (100.0%)</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>0.66</v>
+        <v>2.37</v>
       </c>
       <c r="J4" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>46.15</v>
+        <v>30.43</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>613</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>489</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>79.77</v>
       </c>
       <c r="P4" t="n">
-        <v>366</v>
+        <v>59.23</v>
       </c>
       <c r="Q4" t="n">
-        <v>249</v>
+        <v>160</v>
       </c>
       <c r="R4" t="n">
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="S4" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="T4" t="n">
-        <v>136</v>
+        <v>95</v>
       </c>
       <c r="U4" t="n">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="V4" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="W4" t="n">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="X4" t="n">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="Y4" t="n">
-        <v>32</v>
+        <v>170</v>
       </c>
       <c r="Z4" t="n">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="AA4" t="n">
-        <v>23</v>
+        <v>46.47</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Balcatta - Perth 0:1</t>
+          <t>Perth - Sorrento 3:0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -8259,91 +8259,91 @@
         </is>
       </c>
       <c r="E5" t="n">
+        <v>94</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>4-4-2 (100.0%)</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="J5" t="n">
+        <v>31</v>
+      </c>
+      <c r="K5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" t="n">
+        <v>19.35</v>
+      </c>
+      <c r="M5" t="n">
+        <v>559</v>
+      </c>
+      <c r="N5" t="n">
+        <v>467</v>
+      </c>
+      <c r="O5" t="n">
+        <v>83.54000000000001</v>
+      </c>
+      <c r="P5" t="n">
+        <v>62.54</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>108</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>13</v>
+      </c>
+      <c r="T5" t="n">
+        <v>94</v>
+      </c>
+      <c r="U5" t="n">
         <v>91</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Balcatta</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>4-2-3-1 (49.96%)</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="J5" t="n">
+      <c r="V5" t="n">
         <v>8</v>
       </c>
-      <c r="K5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L5" t="n">
-        <v>50</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="n">
-        <v>416</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>295</v>
-      </c>
-      <c r="R5" t="n">
-        <v>70</v>
-      </c>
-      <c r="S5" t="n">
-        <v>55</v>
-      </c>
-      <c r="T5" t="n">
-        <v>164</v>
-      </c>
-      <c r="U5" t="n">
-        <v>36</v>
-      </c>
-      <c r="V5" t="n">
-        <v>72</v>
-      </c>
       <c r="W5" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="X5" t="n">
-        <v>99</v>
+        <v>45</v>
       </c>
       <c r="Y5" t="n">
-        <v>47</v>
+        <v>179</v>
       </c>
       <c r="Z5" t="n">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="AA5" t="n">
-        <v>17</v>
+        <v>46.93</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Perth - West NTC 3:0</t>
+          <t>Subiaco - Perth 0:5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -8365,78 +8365,78 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>2.37</v>
+        <v>2.25</v>
       </c>
       <c r="J6" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="K6" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="L6" t="n">
-        <v>30.43</v>
+        <v>81.25</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>376</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="O6" t="n">
-        <v>1</v>
+        <v>70.48</v>
       </c>
       <c r="P6" t="n">
-        <v>613</v>
+        <v>55.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>489</v>
+        <v>137</v>
       </c>
       <c r="R6" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="S6" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="T6" t="n">
-        <v>160</v>
+        <v>69</v>
       </c>
       <c r="U6" t="n">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="V6" t="n">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="W6" t="n">
-        <v>95</v>
+        <v>44</v>
       </c>
       <c r="X6" t="n">
-        <v>106</v>
+        <v>22</v>
       </c>
       <c r="Y6" t="n">
-        <v>30</v>
+        <v>242</v>
       </c>
       <c r="Z6" t="n">
-        <v>55</v>
+        <v>126</v>
       </c>
       <c r="AA6" t="n">
-        <v>21</v>
+        <v>52.07</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Perth - West NTC 3:0</t>
+          <t>West NTC - Perth 0:1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -8445,91 +8445,91 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>West NTC</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-4-2 (100.0%)</t>
+          <t>4-1-4-1 (100.0%)</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0.45</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L7" t="n">
-        <v>28.57</v>
+        <v>50</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>596</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>453</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="P7" t="n">
-        <v>401</v>
+        <v>64.13</v>
       </c>
       <c r="Q7" t="n">
-        <v>277</v>
+        <v>176</v>
       </c>
       <c r="R7" t="n">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="S7" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="T7" t="n">
-        <v>172</v>
+        <v>88</v>
       </c>
       <c r="U7" t="n">
-        <v>47</v>
+        <v>121</v>
       </c>
       <c r="V7" t="n">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="W7" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="X7" t="n">
-        <v>106</v>
+        <v>26</v>
       </c>
       <c r="Y7" t="n">
-        <v>59</v>
+        <v>221</v>
       </c>
       <c r="Z7" t="n">
-        <v>42</v>
+        <v>124</v>
       </c>
       <c r="AA7" t="n">
-        <v>5</v>
+        <v>56.11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Perth - Sorrento 3:0</t>
+          <t>Perth - Perth RedStar 1:1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -8538,7 +8538,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -8547,82 +8547,82 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-4-2 (100.0%)</t>
+          <t>4-1-4-1 (100.0%)</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>4.37</v>
+        <v>1.38</v>
       </c>
       <c r="J8" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="K8" t="n">
         <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>19.35</v>
+        <v>54.55</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>386</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>559</v>
+        <v>45.86</v>
       </c>
       <c r="Q8" t="n">
-        <v>467</v>
+        <v>155</v>
       </c>
       <c r="R8" t="n">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="S8" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T8" t="n">
-        <v>108</v>
+        <v>76</v>
       </c>
       <c r="U8" t="n">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="V8" t="n">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="W8" t="n">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="X8" t="n">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="Y8" t="n">
-        <v>8</v>
+        <v>259</v>
       </c>
       <c r="Z8" t="n">
-        <v>38</v>
+        <v>141</v>
       </c>
       <c r="AA8" t="n">
-        <v>45</v>
+        <v>54.44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Perth - Sorrento 3:0</t>
+          <t>UWA Nedlands - Perth 1:3</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -8631,91 +8631,91 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sorrento</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-5-1 (100.0%)</t>
+          <t>4-3-3 (100.0%)</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1.68</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>47.06</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>366</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>68.31</v>
       </c>
       <c r="P9" t="n">
-        <v>284</v>
+        <v>52</v>
       </c>
       <c r="Q9" t="n">
-        <v>178</v>
+        <v>113</v>
       </c>
       <c r="R9" t="n">
+        <v>10</v>
+      </c>
+      <c r="S9" t="n">
+        <v>41</v>
+      </c>
+      <c r="T9" t="n">
         <v>62</v>
       </c>
-      <c r="S9" t="n">
-        <v>37</v>
-      </c>
-      <c r="T9" t="n">
-        <v>140</v>
-      </c>
       <c r="U9" t="n">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="V9" t="n">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="W9" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="X9" t="n">
-        <v>75</v>
+        <v>24</v>
       </c>
       <c r="Y9" t="n">
-        <v>68</v>
+        <v>203</v>
       </c>
       <c r="Z9" t="n">
-        <v>6</v>
+        <v>106</v>
       </c>
       <c r="AA9" t="n">
-        <v>1</v>
+        <v>52.22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Subiaco - Perth 0:5</t>
+          <t>Perth - Balcatta 0:0</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -8724,7 +8724,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -8733,82 +8733,82 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-2-3-1 (100.0%)</t>
+          <t>4-1-4-1 (100.0%)</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>2.25</v>
+        <v>1.24</v>
       </c>
       <c r="J10" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K10" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="L10" t="n">
-        <v>81.25</v>
+        <v>30.77</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>391</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>281</v>
       </c>
       <c r="O10" t="n">
-        <v>2</v>
+        <v>71.87</v>
       </c>
       <c r="P10" t="n">
-        <v>376</v>
+        <v>39.92</v>
       </c>
       <c r="Q10" t="n">
-        <v>265</v>
+        <v>137</v>
       </c>
       <c r="R10" t="n">
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="S10" t="n">
+        <v>60</v>
+      </c>
+      <c r="T10" t="n">
+        <v>60</v>
+      </c>
+      <c r="U10" t="n">
+        <v>115</v>
+      </c>
+      <c r="V10" t="n">
         <v>55</v>
       </c>
-      <c r="T10" t="n">
-        <v>137</v>
-      </c>
-      <c r="U10" t="n">
-        <v>20</v>
-      </c>
-      <c r="V10" t="n">
-        <v>48</v>
-      </c>
       <c r="W10" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="X10" t="n">
-        <v>105</v>
+        <v>23</v>
       </c>
       <c r="Y10" t="n">
-        <v>39</v>
+        <v>200</v>
       </c>
       <c r="Z10" t="n">
-        <v>44</v>
+        <v>98</v>
       </c>
       <c r="AA10" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Subiaco - Perth 0:5</t>
+          <t>Perth - Fremantle City 0:0</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -8821,87 +8821,87 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Subiaco</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3-3 (100.0%)</t>
+          <t>4-2-3-1 (48.4%)</t>
         </is>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0.13</v>
+        <v>0.53</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>516</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>416</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>80.62</v>
       </c>
       <c r="P11" t="n">
-        <v>328</v>
+        <v>51.92</v>
       </c>
       <c r="Q11" t="n">
-        <v>215</v>
+        <v>128</v>
       </c>
       <c r="R11" t="n">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="S11" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="T11" t="n">
-        <v>164</v>
+        <v>57</v>
       </c>
       <c r="U11" t="n">
-        <v>39</v>
+        <v>97</v>
       </c>
       <c r="V11" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="W11" t="n">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="X11" t="n">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="Y11" t="n">
-        <v>41</v>
+        <v>173</v>
       </c>
       <c r="Z11" t="n">
-        <v>36</v>
+        <v>87</v>
       </c>
       <c r="AA11" t="n">
-        <v>12</v>
+        <v>50.29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>West NTC - Perth 0:1</t>
+          <t>Sorrento - Perth 0:2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8910,7 +8910,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -8923,78 +8923,78 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>1.84</v>
       </c>
       <c r="J12" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="K12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L12" t="n">
-        <v>50</v>
+        <v>26.67</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>372</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>78.81</v>
       </c>
       <c r="P12" t="n">
-        <v>596</v>
+        <v>59.94</v>
       </c>
       <c r="Q12" t="n">
-        <v>453</v>
+        <v>112</v>
       </c>
       <c r="R12" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="S12" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="T12" t="n">
-        <v>176</v>
+        <v>67</v>
       </c>
       <c r="U12" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="V12" t="n">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="W12" t="n">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="X12" t="n">
+        <v>27</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>198</v>
+      </c>
+      <c r="Z12" t="n">
         <v>121</v>
       </c>
-      <c r="Y12" t="n">
-        <v>32</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>63</v>
-      </c>
       <c r="AA12" t="n">
-        <v>26</v>
+        <v>61.11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>West NTC - Perth 0:1</t>
+          <t>Perth - Subiaco 2:0</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -9003,91 +9003,91 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>West NTC</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-4-2 (100.0%)</t>
+          <t>4-2-3-1 (100.0%)</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>0.38</v>
+        <v>1.74</v>
       </c>
       <c r="J13" t="n">
+        <v>18</v>
+      </c>
+      <c r="K13" t="n">
         <v>8</v>
       </c>
-      <c r="K13" t="n">
-        <v>4</v>
-      </c>
       <c r="L13" t="n">
-        <v>50</v>
+        <v>44.44</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>429</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>308</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>71.79000000000001</v>
       </c>
       <c r="P13" t="n">
-        <v>311</v>
+        <v>50.98</v>
       </c>
       <c r="Q13" t="n">
-        <v>188</v>
+        <v>167</v>
       </c>
       <c r="R13" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="S13" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="T13" t="n">
-        <v>183</v>
+        <v>78</v>
       </c>
       <c r="U13" t="n">
-        <v>34</v>
+        <v>106</v>
       </c>
       <c r="V13" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="W13" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="X13" t="n">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="Y13" t="n">
-        <v>50</v>
+        <v>170</v>
       </c>
       <c r="Z13" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="AA13" t="n">
-        <v>12</v>
+        <v>47.65</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Perth - Perth RedStar 1:1</t>
+          <t>Perth - UWA Nedlands 6:0</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -9096,7 +9096,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -9105,1277 +9105,68 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-1-4-1 (100.0%)</t>
+          <t>4-3-3 (100.0%)</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I14" t="n">
-        <v>1.38</v>
+        <v>1.77</v>
       </c>
       <c r="J14" t="n">
+        <v>20</v>
+      </c>
+      <c r="K14" t="n">
         <v>11</v>
       </c>
-      <c r="K14" t="n">
-        <v>6</v>
-      </c>
       <c r="L14" t="n">
-        <v>54.55</v>
+        <v>55</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>514</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>411</v>
       </c>
       <c r="O14" t="n">
-        <v>1</v>
+        <v>79.95999999999999</v>
       </c>
       <c r="P14" t="n">
-        <v>386</v>
+        <v>62.41</v>
       </c>
       <c r="Q14" t="n">
-        <v>280</v>
+        <v>132</v>
       </c>
       <c r="R14" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="S14" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="T14" t="n">
+        <v>101</v>
+      </c>
+      <c r="U14" t="n">
+        <v>95</v>
+      </c>
+      <c r="V14" t="n">
+        <v>19</v>
+      </c>
+      <c r="W14" t="n">
+        <v>44</v>
+      </c>
+      <c r="X14" t="n">
+        <v>32</v>
+      </c>
+      <c r="Y14" t="n">
         <v>155</v>
       </c>
-      <c r="U14" t="n">
-        <v>19</v>
-      </c>
-      <c r="V14" t="n">
-        <v>60</v>
-      </c>
-      <c r="W14" t="n">
-        <v>76</v>
-      </c>
-      <c r="X14" t="n">
-        <v>120</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>47</v>
-      </c>
       <c r="Z14" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="AA14" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>7</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Perth - Perth RedStar 1:1</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>96</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Perth RedStar</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>4-4-2 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="J15" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" t="n">
-        <v>16.67</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
-        <v>420</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>315</v>
-      </c>
-      <c r="R15" t="n">
-        <v>75</v>
-      </c>
-      <c r="S15" t="n">
-        <v>54</v>
-      </c>
-      <c r="T15" t="n">
-        <v>157</v>
-      </c>
-      <c r="U15" t="n">
-        <v>21</v>
-      </c>
-      <c r="V15" t="n">
-        <v>68</v>
-      </c>
-      <c r="W15" t="n">
-        <v>68</v>
-      </c>
-      <c r="X15" t="n">
-        <v>105</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>44</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>46</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>UWA Nedlands - Perth 1:3</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>93</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Perth</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>4-3-3 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>3</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="J16" t="n">
-        <v>17</v>
-      </c>
-      <c r="K16" t="n">
-        <v>8</v>
-      </c>
-      <c r="L16" t="n">
-        <v>47.06</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>366</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>250</v>
-      </c>
-      <c r="R16" t="n">
-        <v>68</v>
-      </c>
-      <c r="S16" t="n">
-        <v>52</v>
-      </c>
-      <c r="T16" t="n">
-        <v>113</v>
-      </c>
-      <c r="U16" t="n">
-        <v>10</v>
-      </c>
-      <c r="V16" t="n">
-        <v>41</v>
-      </c>
-      <c r="W16" t="n">
-        <v>62</v>
-      </c>
-      <c r="X16" t="n">
-        <v>92</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>29</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>39</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>8</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>UWA Nedlands - Perth 1:3</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>93</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>UWA Nedlands</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>4-2-3-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="J17" t="n">
-        <v>4</v>
-      </c>
-      <c r="K17" t="n">
-        <v>4</v>
-      </c>
-      <c r="L17" t="n">
-        <v>100</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>281</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>185</v>
-      </c>
-      <c r="R17" t="n">
-        <v>65</v>
-      </c>
-      <c r="S17" t="n">
-        <v>48</v>
-      </c>
-      <c r="T17" t="n">
-        <v>150</v>
-      </c>
-      <c r="U17" t="n">
-        <v>33</v>
-      </c>
-      <c r="V17" t="n">
-        <v>67</v>
-      </c>
-      <c r="W17" t="n">
-        <v>50</v>
-      </c>
-      <c r="X17" t="n">
-        <v>75</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>40</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>31</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>9</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Perth - Balcatta 0:0</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>99</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Perth</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>4-1-4-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="J18" t="n">
-        <v>13</v>
-      </c>
-      <c r="K18" t="n">
-        <v>4</v>
-      </c>
-      <c r="L18" t="n">
-        <v>30.77</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="n">
-        <v>2</v>
-      </c>
-      <c r="P18" t="n">
-        <v>391</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>281</v>
-      </c>
-      <c r="R18" t="n">
-        <v>71</v>
-      </c>
-      <c r="S18" t="n">
-        <v>39</v>
-      </c>
-      <c r="T18" t="n">
-        <v>137</v>
-      </c>
-      <c r="U18" t="n">
-        <v>17</v>
-      </c>
-      <c r="V18" t="n">
-        <v>60</v>
-      </c>
-      <c r="W18" t="n">
-        <v>60</v>
-      </c>
-      <c r="X18" t="n">
-        <v>115</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>55</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>37</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>9</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Perth - Balcatta 0:0</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>99</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Balcatta</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>4-4-1-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="J19" t="n">
-        <v>10</v>
-      </c>
-      <c r="K19" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" t="n">
-        <v>40</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P19" t="n">
-        <v>503</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>371</v>
-      </c>
-      <c r="R19" t="n">
-        <v>73</v>
-      </c>
-      <c r="S19" t="n">
-        <v>60</v>
-      </c>
-      <c r="T19" t="n">
-        <v>162</v>
-      </c>
-      <c r="U19" t="n">
-        <v>31</v>
-      </c>
-      <c r="V19" t="n">
-        <v>52</v>
-      </c>
-      <c r="W19" t="n">
-        <v>79</v>
-      </c>
-      <c r="X19" t="n">
-        <v>104</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>41</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>53</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Perth - Fremantle City 0:0</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>95</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Perth</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-2-3-1 (48.4%)</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="J20" t="n">
-        <v>10</v>
-      </c>
-      <c r="K20" t="n">
-        <v>3</v>
-      </c>
-      <c r="L20" t="n">
-        <v>30</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>516</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>416</v>
-      </c>
-      <c r="R20" t="n">
-        <v>80</v>
-      </c>
-      <c r="S20" t="n">
-        <v>51</v>
-      </c>
-      <c r="T20" t="n">
-        <v>128</v>
-      </c>
-      <c r="U20" t="n">
-        <v>18</v>
-      </c>
-      <c r="V20" t="n">
-        <v>53</v>
-      </c>
-      <c r="W20" t="n">
-        <v>57</v>
-      </c>
-      <c r="X20" t="n">
-        <v>97</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>54</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>32</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>10</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Perth - Fremantle City 0:0</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>95</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Fremantle City</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-2-3-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="n">
-        <v>1</v>
-      </c>
-      <c r="P21" t="n">
-        <v>417</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>314</v>
-      </c>
-      <c r="R21" t="n">
-        <v>75</v>
-      </c>
-      <c r="S21" t="n">
-        <v>48</v>
-      </c>
-      <c r="T21" t="n">
-        <v>144</v>
-      </c>
-      <c r="U21" t="n">
-        <v>26</v>
-      </c>
-      <c r="V21" t="n">
-        <v>35</v>
-      </c>
-      <c r="W21" t="n">
-        <v>83</v>
-      </c>
-      <c r="X21" t="n">
-        <v>79</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>36</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>38</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>11</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Sorrento - Perth 0:2</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>94</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Perth</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-1-4-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H22" t="n">
-        <v>2</v>
-      </c>
-      <c r="I22" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="J22" t="n">
-        <v>30</v>
-      </c>
-      <c r="K22" t="n">
-        <v>8</v>
-      </c>
-      <c r="L22" t="n">
-        <v>26.67</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="n">
-        <v>472</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>372</v>
-      </c>
-      <c r="R22" t="n">
-        <v>78</v>
-      </c>
-      <c r="S22" t="n">
-        <v>59</v>
-      </c>
-      <c r="T22" t="n">
-        <v>112</v>
-      </c>
-      <c r="U22" t="n">
-        <v>10</v>
-      </c>
-      <c r="V22" t="n">
-        <v>35</v>
-      </c>
-      <c r="W22" t="n">
-        <v>67</v>
-      </c>
-      <c r="X22" t="n">
-        <v>100</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>19</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>54</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Sorrento - Perth 0:2</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>94</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Sorrento</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>4-5-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J23" t="n">
-        <v>7</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>28.57</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="n">
-        <v>1</v>
-      </c>
-      <c r="P23" t="n">
-        <v>316</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>221</v>
-      </c>
-      <c r="R23" t="n">
-        <v>69</v>
-      </c>
-      <c r="S23" t="n">
-        <v>40</v>
-      </c>
-      <c r="T23" t="n">
-        <v>134</v>
-      </c>
-      <c r="U23" t="n">
-        <v>38</v>
-      </c>
-      <c r="V23" t="n">
-        <v>68</v>
-      </c>
-      <c r="W23" t="n">
-        <v>28</v>
-      </c>
-      <c r="X23" t="n">
-        <v>72</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>44</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>20</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>12</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-03-29</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Perth - Subiaco 2:0</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>96</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Perth</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>4-2-3-1 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>2</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="J24" t="n">
-        <v>18</v>
-      </c>
-      <c r="K24" t="n">
-        <v>8</v>
-      </c>
-      <c r="L24" t="n">
-        <v>44.44</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
-        <v>429</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>308</v>
-      </c>
-      <c r="R24" t="n">
-        <v>71</v>
-      </c>
-      <c r="S24" t="n">
-        <v>50</v>
-      </c>
-      <c r="T24" t="n">
-        <v>167</v>
-      </c>
-      <c r="U24" t="n">
-        <v>38</v>
-      </c>
-      <c r="V24" t="n">
-        <v>51</v>
-      </c>
-      <c r="W24" t="n">
-        <v>78</v>
-      </c>
-      <c r="X24" t="n">
-        <v>106</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>51</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>44</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>12</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-03-29</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Perth - Subiaco 2:0</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>96</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Subiaco</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>4-4-2 (49.52%)</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>1.31</v>
-      </c>
-      <c r="J25" t="n">
-        <v>15</v>
-      </c>
-      <c r="K25" t="n">
-        <v>3</v>
-      </c>
-      <c r="L25" t="n">
-        <v>20</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>1</v>
-      </c>
-      <c r="P25" t="n">
-        <v>382</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>260</v>
-      </c>
-      <c r="R25" t="n">
-        <v>68</v>
-      </c>
-      <c r="S25" t="n">
-        <v>49</v>
-      </c>
-      <c r="T25" t="n">
-        <v>154</v>
-      </c>
-      <c r="U25" t="n">
-        <v>21</v>
-      </c>
-      <c r="V25" t="n">
-        <v>68</v>
-      </c>
-      <c r="W25" t="n">
-        <v>65</v>
-      </c>
-      <c r="X25" t="n">
-        <v>94</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>46</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>26</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>13</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Perth - UWA Nedlands 6:0</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>95</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Perth</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>4-3-3 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H26" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="J26" t="n">
-        <v>20</v>
-      </c>
-      <c r="K26" t="n">
-        <v>11</v>
-      </c>
-      <c r="L26" t="n">
-        <v>55</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="n">
-        <v>1</v>
-      </c>
-      <c r="P26" t="n">
-        <v>514</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>411</v>
-      </c>
-      <c r="R26" t="n">
-        <v>79</v>
-      </c>
-      <c r="S26" t="n">
-        <v>62</v>
-      </c>
-      <c r="T26" t="n">
-        <v>132</v>
-      </c>
-      <c r="U26" t="n">
-        <v>4</v>
-      </c>
-      <c r="V26" t="n">
-        <v>27</v>
-      </c>
-      <c r="W26" t="n">
-        <v>101</v>
-      </c>
-      <c r="X26" t="n">
-        <v>95</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>19</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>44</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>13</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Perth - UWA Nedlands 6:0</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Australia. Western Australia NPL Women</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>95</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>UWA Nedlands</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>3-5-2 (100.0%)</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J27" t="n">
-        <v>4</v>
-      </c>
-      <c r="K27" t="n">
-        <v>2</v>
-      </c>
-      <c r="L27" t="n">
-        <v>50</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>319</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>229</v>
-      </c>
-      <c r="R27" t="n">
-        <v>71</v>
-      </c>
-      <c r="S27" t="n">
-        <v>37</v>
-      </c>
-      <c r="T27" t="n">
-        <v>126</v>
-      </c>
-      <c r="U27" t="n">
-        <v>43</v>
-      </c>
-      <c r="V27" t="n">
-        <v>62</v>
-      </c>
-      <c r="W27" t="n">
-        <v>21</v>
-      </c>
-      <c r="X27" t="n">
-        <v>80</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>48</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>31</v>
-      </c>
-      <c r="AA27" t="n">
-        <v>1</v>
+        <v>50.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização semanal — Round 14
</commit_message>
<xml_diff>
--- a/team_stats_perth.xlsx
+++ b/team_stats_perth.xlsx
@@ -8626,7 +8626,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -8719,7 +8719,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -8812,7 +8812,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -8905,7 +8905,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -9091,7 +9091,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -9184,7 +9184,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -9277,7 +9277,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -9370,7 +9370,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -9463,7 +9463,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -9556,7 +9556,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -9649,7 +9649,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -9742,7 +9742,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -9928,7 +9928,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -10114,7 +10114,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -10207,7 +10207,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -10300,7 +10300,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -10486,7 +10486,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -10579,7 +10579,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -10672,7 +10672,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -10765,7 +10765,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -10858,7 +10858,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -10951,7 +10951,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -11044,7 +11044,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>

</xml_diff>